<commit_message>
corrected the mcmc configuration content
</commit_message>
<xml_diff>
--- a/inst/extdata/default_mcmc_config.xlsx
+++ b/inst/extdata/default_mcmc_config.xlsx
@@ -1,68 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/24b25e554f22146a/Masters Class notes/AIMS Rwanda/Thesis Phase/Publication Phase/Code Test/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="38" documentId="11_22D3943CEC27AC06FF42925F060A5312A27FC05C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2930F479-A240-4197-8362-45051FAD3D1E}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="2160" yWindow="2160" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="params" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
-  <si>
-    <t>parameter</t>
-  </si>
-  <si>
-    <t>value</t>
-  </si>
-  <si>
-    <t>n_chains</t>
-  </si>
-  <si>
-    <t>chunk_size</t>
-  </si>
-  <si>
-    <t>max_iterations</t>
-  </si>
-  <si>
-    <t>burn_in_frac</t>
-  </si>
-  <si>
-    <t>rhat_threshold</t>
-  </si>
-  <si>
-    <t>ess_threshold</t>
-  </si>
-  <si>
-    <t>record_hidden_alleles</t>
-  </si>
-  <si>
-    <t>thinning_interval</t>
-  </si>
-  <si>
-    <t>random_seed</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -88,27 +52,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -157,6 +112,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -182,12 +141,15 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -213,7 +175,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -389,95 +350,73 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="19.109375" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>2</v>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>parameter</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>n_chains</t>
+        </is>
       </c>
       <c r="B2">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>3</v>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>iter</t>
+        </is>
       </c>
       <c r="B3">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>4</v>
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>burn_in_frac</t>
+        </is>
       </c>
       <c r="B4">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>5</v>
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>random_seed</t>
+        </is>
       </c>
       <c r="B5">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>6</v>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>adapt_delta</t>
+        </is>
       </c>
       <c r="B6">
-        <v>1.1000000000000001</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10">
-        <v>42</v>
+        <v>0.85</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>